<commit_message>
Bring Prepared_Dataset and KB updates from final-data-update
Copy from origin/final-data-update@cdf1d8da:
- Prepared_Dataset: 9 crops + metadata (Banana, Cauliflower, Coffee,
  Corn, Orange, Soybean, Sugarcane, Tomato, Wheat). Mango_Leaf and
  Mango_Leaf_test preserved from main (not on final-data-update).
- disease_registry/outputs (KB): Banana, Cauliflower, Coffee, Orange,
  Sugarcane, Tomato, Wheat plus tag_image_raw.txt. Soybean, Corn,
  Mango_Leaf KBs left at main's versions per request.

Code (run_sweeps.sh, pipeline.py, run_sweeps_available.sh, pyc files)
intentionally not pulled.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/disease_registry/outputs/Tomato/internet.xlsx
+++ b/disease_registry/outputs/Tomato/internet.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Disease Registry" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Disease Registry" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,27 +456,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Leaf_Mold</t>
+          <t>Cucumber_Mosaic_Virus</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Passalora fulva</t>
+          <t>Cucumber mosaic virus</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Blossom, Fruit</t>
+          <t>Foliar, Stem, Vascular, Whole plant, Seed</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pale greenish-yellow spots, usually less than 1/4 inch with no definite margins, form on the upper sides of leaves. Olive-green to brown velvety mold forms on the lower leaf surface below leaf spots. Leaves wither and die but often remain attached to the plant.. Discrete yellow spots on the upper side of the leaf with corresponding olive-colored velvety spores (conidia) on the underside; oldest leaves infected first with disease progressing upward; fruit infections appear as a smooth black irregular area at the stem end that becomes sunken, dry, and leathery.. Magnesium deficiency, Nutrient deficiency (general), Early stages of other diseases</t>
+          <t>CMV causes stunting, mosaic patterns of light and dark green or yellow and green on leaves, malformation of leaves and growing points, yellow streaking and spotting, ring-spots or line patterns on leaves or fruit, flower color breaking, and yellowing of veins.. Alternating light and dark green mosaic pattern on leaves, especially younger leaves, with possible shoestring-like appearance of leaves; plants appear lighter in color, bushy and stunted.. Tobacco mosaic virus</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -485,38 +485,34 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tomato_Yellow_Leaf_Curl_Virus</t>
+          <t>Early_Blight</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tomato yellow leaf curl virus</t>
+          <t>Alternaria solani</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Viral</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Foliar, Stem, Whole plant</t>
-        </is>
-      </c>
+          <t>Fungal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Infected plants show small, upward-curling leaves with strong crumpling and interveinal and marginal yellowing, accompanied by stunted, bushy growth due to shortened internodes. Plants may also exhibit flower drop and dramatically reduced fruit production.. Characteristic 'bonsai' or 'broccoli'-like bushy appearance due to shortened internodes combined with small, upward-curling leaves showing interveinal and marginal yellowing; chlorosis first appears on young leaves; plants infected with TYLCV appear patchy across the field rather than uniformly affected; flowers commonly abscise and fruit production is dramatically reduced.. potassium deficiency, magnesium deficiency, micronutrient deficiencies, leaf curl, excessive aphid feeding, other viruses</t>
+          <t>Lesions are larger and darker brown than Septoria leaf spots and display concentric rings.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -526,12 +522,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Early_Blight</t>
+          <t>Gray_Mold</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alternaria linariae</t>
+          <t>Botrytis cinerea</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -541,12 +537,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Pod</t>
+          <t>Foliar, Stem, Fruit, Pod</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Roughly circular brown spots appear on leaves and stems, enlarging to show concentric rings giving a target-like appearance, often with a yellow halo; multiple spots can merge causing extensive leaf tissue destruction and total defoliation of lower leaves. Lesions on fruit are typically sunken, leathery, and dark brown to black with concentric rings.. Large brownish-black lesions with characteristic concentric rings giving a target-like appearance, often surrounded by a yellow halo; symptoms begin at the base of the plant on lower leaves; lesions can expand to about 1/4–1/2 inch in diameter.. Septoria leaf spot, Gray leaf spot, Late blight, Bacterial spot</t>
+          <t>Botrytis produces a dense velvety gray-brown spore mass on infected tissue. Lesions on leaves and stems are tan to brown in color. In high humidity, fluffy gray spores cover infected plant parts. Fruit lesions appear as a whitish soft rot with characteristic small white rings (ghost spots) of 3–8 mm on the fruit surface representing aborted infections.. Dense velvety gray-brown spore mass that releases a cloud of spores when disturbed; stem lesions may expand in concentric rings to girdle the entire stem causing wilting above the infection site; spores are light brown-gray on black stalks; characteristic 3–8 mm whitish ghost spot rings on fruit surface; leaves show irregular to V-shaped brown blotches often starting at margins.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -561,27 +557,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bacterial_Spot</t>
+          <t>Late_Blight</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Xanthomonas euvesicatoria, Xanthomonas gardneri, Xanthomonas perforans, Xanthomonas vesicatoria</t>
+          <t>Phytophthora infestans</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Oomycete</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Pod</t>
+          <t>Foliar, Stem, Fruit, Flowers, Whole plant</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>On tomato, leaf lesions are initially circular and water-soaked, may be surrounded by a faint yellow halo, and are dark brown to black. Fruit lesions begin as small, slightly raised blisters that become dark brown and scab-like.. Leaf lesions are initially circular and water-soaked with a wet or greasy appearance, may develop a faint halo that later disappears, and rarely exceed 3 mm in diameter. In X. perforans infections, dead tissue in lesion centers can drop out giving a 'shot hole' appearance. Bacterial streaming (ooze) observable under a light microscope from excised lesions distinguishes this from fungal diseases. Tomato leaf spots lack concentric rings and have yellow halos with centers that fall out; tomato fruit spots have a waxy white halo. Pepper leaf spots lack yellow halos and centers do not fall out.. bacterial speck, early blight, gray leaf spot, target spot, Septoria leaf spot</t>
+          <t>Infected leaves develop green to brown patches of dead tissue surrounded by a pale green or gray border; under humid and wet conditions, lesions appear water-soaked, dark brown, and greasy, with white fuzzy growth on undersides of leaves and lower stems. Stem and petiole lesions are brown and not well-defined in shape. Flowers may discolor and drop. Fruit lesions appear as firm, greasy spots that become leathery and chocolate brown, or mottled with golden to dark brown firm sunken surfaces with associated white fuzzy pathogen growth.. White fuzzy pathogen sporulation visible on undersides of leaves and lower stems; lesions are brown and papery with rings of white fuzzy sporulation; leaf lesions surrounded by distinctive pale green or gray halos; water-soaked or greasy appearance under humid conditions; late blight lesions found anywhere on plant (especially new growth) and are light brown or tan, distinguishing them from early blight (dark brown with concentric rings, starting on lower leaves).. Phytophthora nicotianae, Phytophthora capsici, Early blight</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -596,32 +592,32 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Late_Blight</t>
+          <t>Bacterial_Canker_And_Wilt_Of_Tomato</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Phytophthora infestans</t>
+          <t>Clavibacter michiganensis subsp. michiganensis</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Oomycete</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Pod</t>
+          <t>Foliar, Stem, Fruit</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Leaf symptoms first appear as small, water-soaked areas that rapidly enlarge to form purple-brown, oily-appearing blotches; during high humidity, white cottony growth (sporangia) appears on the underside of leaves. Infected fruit turn brown and firm with greasy spots that eventually become leathery and chocolate brown, symptoms typically beginning on the shoulders of the fruit.. Grayish white mycelium and spore-forming structures appear on the lower side of leaves around purple-brown blotches; lesions are mostly found on new growth and tend to be light brown or tan in color; white cottony sporulation visible on leaf undersides during high humidity.. Phytophthora nicotianae, Phytophthora capsici, Early blight</t>
+          <t>Symptoms include wilting, defoliation, and desiccation of leaves, along with brown canker lesions on stems and fruit marked by characteristic dark spots surrounded by white halos.. The bird-eye spots on the fruit are small dark brown lesions that are surrounded by a white halo and may become raised as symptoms progress, with scorching and browning of leaf margins. Bacterial canker can be distinguished from bacterial speck by excessive wilting, canker development, and prominent bird's-eye spots on fruit.. Bacterial Speck, Bacterial Spot</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -631,12 +627,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bacterial_Leaf_Spot</t>
+          <t>Bacterial_Speck_Of_Tomato</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Xanthomonas euvesicatoria, Xanthomonas vesicatoria, Xanthomonas perforans, Xanthomonas gardneri</t>
+          <t>Pseudomonas syringae pv. tomato</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -646,102 +642,102 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Foliar, Pod</t>
+          <t>Foliar, Fruit</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bacterial leaf spot causes leaf lesions with yellowing and large crusty spots on the fruit, leading to non-marketable tomatoes.. Leaf lesions with yellowing and large crusty spots on fruit.. Bacterial Canker, Bacterial Speck of Tomato, Septoria Leaf Spot</t>
+          <t>Small black spots with yellow halos on leaves and fruit. On leaves, spots are 1/8 to 1/4 inch in diameter, angular, and more prominent on undersides; on fruit, spots are pinpoint-like, slightly raised, and can be raised, flat, or sunken, ranging from brown to black.. Small (1/16 in.) slightly-raised black speck-like lesions on developing fruit much smaller than those of bacterial spot; on leaves, small angular (straight-edged) spots with yellow halos; substantial leaf curling may also be present.. Bacterial Spot of Tomato, Bacterial Canker, Tomato Spotted Wilt, Bacterial Leaf Spot</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tomato_Mosaic_Virus</t>
+          <t>Southern_Bacterial_Wilt</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tomato mosaic virus</t>
+          <t>Ralstonia solanacearum Race 1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Foliar, Pod, Seed, Whole plant</t>
+          <t>Root, Stem, Vascular, Whole plant</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Infected tomato plants show a mosaic pattern on leaves with blotchy light and dark spots; leaves may develop yellow streaks or spots and become malformed; fruit may ripen unevenly with deformation; early infection may cause yellowing and stunting; fruits may also show irregular off-color spots (elevated or depressed) and browning just beneath the skin (brownwall).. Dark and light green mottling on leaves combined with fruit browning just beneath the skin (brownwall) and irregular, off-color spots on fruit that can be either elevated or depressed; visually very similar to TMV and distinguished mainly by host preference (primarily tomato).. Tobacco Mosaic Virus (TMV), Tomato Brown Rugose Fruit Virus (ToBRFV), Herbicide injury, Other tomato viruses</t>
+          <t>Initially, infected plants develop wilt symptoms in the afternoon and recover in the evening. As the disease progresses, the base of the plant shows brown cankers and root rot with vascular discoloration, eventually leading to permanent wilt and plant death.. A white slimy bacterial substance streams from a freshly cut stem base placed in water, which is a strong indicator of bacteria in the vascular tissue. The interior stem shows dark or light brown discoloration in the pith area.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Powdery_Mildew</t>
+          <t>Tomato_Spotted_Wilt_Virus</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Oidium neolycopersici</t>
+          <t>Tomato spotted wilt virus (TSWV)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fungal</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Foliar</t>
+          <t>Foliar, Fruit, Whole plant</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Symptoms appear on foliage as light-green to bright yellow lesions on the upper leaf surface that enlarge and become necrotic, with a light powdery coating visible on leaf undersides and potentially a dense white layer of growth on both surfaces; entire leaves wither and die but remain attached to the stem.. White, powdery sporulation on both the tops and undersides of leaves, in round spots that begin small but expand and converge; entire leaves wither and die but remain attached to the stem; no symptoms on fruit or stems.. Early blight</t>
+          <t>Infected leaves appear bronzed with small brown lesions or necrotic spots; infected foliage may become covered with so many spots that leaves brown, roll, and wilt. Fruit develops yellow ringspots and brown necrotic sunken areas. Young leaves develop bronzing on upper surfaces followed by distinct necrotic spots, with leaves cupping downward and tip dieback. Ripe fruit shows chlorotic spots and blotches with concentric rings; green fruit shows slightly raised areas with faint concentric zones.. Lesions caused by TSWV have blurred margins, whereas lesions from other diseases have definite margins. Bronzing on upper leaf surfaces, distinct necrotic spots, downward-cupped leaves, tip dieback, and concentric ring patterns on ripe fruit or raised zones on green fruit are key diagnostic features.. early blight, other leaf spot diseases, other plant viruses</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Septoria_Leaf_Spot</t>
+          <t>Alternaria_Black_Molds_Stem_Cankers</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Septoria lycopersici</t>
+          <t>Alternaria alternata f. sp. lycopersici</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -751,12 +747,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Stem, Foliar, Vascular</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Circular, tan to gray lesions develop on lower leaves and stems; lesions are typically small (&lt;1/8 in) with a dark-brown perimeter, and a yellow halo may develop around leaf lesions. Small dark spots (pycnidia) may appear in the center of the lesion. Multiple spots on a single leaf may merge, leading to extensive destruction of leaf tissue and potential total defoliation.. Small (&lt;1/8 in) circular lesions with a tan to gray center, dark-brown perimeter, possible yellow halo, and small dark pycnidia (fungal fruiting bodies) visible in the center upon close inspection; underside of leaves may appear darker green or water-soaked.. Early blight, Gray leaf spot, Late Blight, Bacterial Speck of Tomato, Bacterial Spot of Tomato</t>
+          <t>Alternaria stem canker is characterized by large, irregularly shaped, dark-brown to almost black cankers with light and dark concentric rings on stems near the soil line, enlarging to cause girdled stems, stem death, and plant collapse.. Alternaria stem canker causes large, irregularly shaped stem lesions with pronounced concentric rings. Vascular and pith tissue directly above and below cankers develop brown streaks and become cracked and dry. Spores are formed in chains of 3-5, light olive brown to dark brown, hand grenade-shaped with a shorter beaked apical cell on the terminal end, and are 7-18 x 18-50 µm in size.. Collar rot</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -765,45 +761,53 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Spider_Mites</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
+          <t>Anthracnose</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Colletotrichum coccodes</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Fungal</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Foliar</t>
+          <t>Foliar, Stem, Root, Pod</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Spider mites cause yellowish to bronze stippling or speckling on leaves, with severe infestations turning entire leaves yellow. Webbing is typically present on the underside of leaves.. Webbing on the underside of leaves, with mites visible as 'moving dust' in the webbing; symptoms worsen in hot, dry, dusty conditions.</t>
+          <t>Anthracnose initially appears as small, circular, water-soaked and sunken spots on overripe tomatoes. These lesions form concentric rings, expand to ½" in diameter, darken progressively, and may merge to cause complete fruit decay. Leaf symptoms appear as small, dark spots surrounded by a yellow halo on older leaves. During damp weather, masses of salmon-colored spores may develop on lesion surfaces.. Dark fungal structures visible in the center of spots; salmon pink spore appearance under humid conditions; concentric ring pattern with tan center and dark specks; water-soaked and sunken lesions expanding to approximately ½" in diameter.. Blossom End Rot, Late Blight</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Verticillium_Wilt</t>
+          <t>Leaf_Mold</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verticillium dahliae and Verticillium albo-atrum</t>
+          <t>Passalora fulva</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -813,12 +817,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Foliar, Vascular, Stem, Root, Whole plant</t>
+          <t>Foliar, Fruit</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Initial symptoms include yellowing of lower leaves, wilting, stunted growth, and V-shaped lesions extending inward from leaf margins. Brown necrotic tissue develops within lesions as disease progresses; lower leaves die and fall off; longitudinal light brown to cream-colored streaks appear beneath the outer stem tissue. Symptoms may appear on only one side of the plant, a branch, or individual leaflets.. V-shaped leaf lesions distinctive of Verticillium wilt; vascular streaking within the stem (light brown to cream-colored longitudinal streaks beneath outer stem tissue, most prominent at the base); vascular streaking in leaves; one-sided symptom expression on a plant, branch, or leaflets; brown vascular discoloration visible when stem is cut lengthwise; symptoms associated with cooler temperatures (68–74°F).. Fusarium wilt, bacterial wilt, southern blight, lack of moisture / insufficient moisture</t>
+          <t>Pale greenish-yellow spots on the upper leaf surface with olive-green to brown velvety mold on the lower surface. Infected leaves eventually wither and die. Fruit infections appear as smooth black irregular areas on the stem end.. Discrete yellow spots on upper leaf surface with corresponding olive spores on underside; oldest leaves infected first; velvety mold texture on lower leaf surface; spots typically less than 1/4 inch with no definite margins. Lesions appear as brighter yellow with indistinct chlorosis on upper leaf surface, underside shows olive-green fuzzy fungal growth.. Cercospora leaf mold</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -827,49 +831,53 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Spider_Mites_Two-Spotted_Spider_Mite</t>
+          <t>Powdery_Mildew</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tetranychus urticae</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>Oidium neolycopersici</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Fungal</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Foliar, Stem</t>
+          <t>Foliar</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Adult TSSM feed by sucking chlorophyll out of the leaves, creating blotchy pale to reddish-brown spots. Feeding injury often gives the top leaf surfaces a mottled or speckled, dull appearance. Leaves then turn yellow and drop. Large populations produce visible webbing that can completely cover the leaves.. Visible webbing covering leaves with mites hiding underneath; adult females are approximately 1/50-inch long, slightly orange or pale green with two dark spots on their body, found predominantly on the undersides of leaves. Check undersides of leaves for tiny black specks of debris and slow-moving mites with a hand lens; shake stems over paper or cloth tray and watch for tiny moving dots.. drought stress</t>
+          <t>Light-green to bright yellow lesions appear on leaf surfaces with white powdery coating, eventually forming a dense white layer of growth that can cover entire leaves. Leaves wither and die while remaining attached to the stem.. White powdery sporulation in round spots that begin small but expand and converge, with light-green to bright yellow lesions that become necrotic, and affected leaves withering and dying while remaining attached to the stem. Lesions may exhibit concentric rings.. Early blight, Leveillula taurica powdery mildew</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Target_Spot</t>
+          <t>Verticillium_Wilt</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Corynespora cassiicola</t>
+          <t>Verticillium dahliae and Verticillium albo-atrum</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -879,141 +887,233 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Foliar, Stem, Root, Fruit</t>
+          <t>Foliar, Vascular</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Leaf lesions start as dark brown pinpoint spots that enlarge with light brown to gray centers and dark concentric rings, sometimes surrounded by yellowing. Fruit lesions begin as small brown sunken flecks that expand into deeply pitted lesions with a characteristic 'X' or star-shaped cracking pattern. Disease typically begins on older lower leaves and progresses upward.. Enlarging lesions develop light brown to gray centers with dark outer concentric rings, sometimes with surrounding chlorosis. Fruit show deeply pitted lesions with a characteristic 'X' or star-shaped cracking pattern. Stem and petiole lesions are dark brown and oval-shaped. Disease typically initiates within the inner canopy and progresses outward. Larger spots can reach up to 10 mm with ring or concentric circle patterns.. early bacterial spot (Xanthomonas spp.), early blight (Alternaria spp.), gray leaf spot (Stemphylium spp.), leaf spot</t>
+          <t>Yellowing of lower leaves followed by wilting, with characteristic V-shaped leaf lesions containing brown necrotic tissue surrounded by irregular yellowing.. V-shaped leaf lesions widest at the leaf margin, brown necrotic tissue surrounded by irregular yellowing, brown vascular discoloration visible when stems are cut lengthwise, and one-sided wilting due to asymmetric vascular colonization.. Fusarium wilt</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Early_Blight_Leaf</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+          <t>Sclerotinia_Timber_Rot</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sclerotinia sclerotiorum</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Fungal</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Stem</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Water-soaked areas develop on the stem that become covered with white cotton-like mycelium, bleached and hardened, eventually causing wilting, collapse, and plant death.. Hard, grayish-black sclerotia about the size of a plump grain of rice embedded within the stem tissue; positive identification achieved by slicing the diseased stem longitudinally.</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Leaf_Bacterial_Spot</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
+          <t>Rhizopus_Soft_Rots</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Rhizopus microsporus</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Fungal</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Soft, watery, slightly sunken lesions accompanied by progressive growth of whitish-gray mycelia with black sporangia, eventually leading to overall decay of infected commodities.. Soft, watery lesions with whitish-gray mycelia and black sporangia.</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Leaf_Late_Blight</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+          <t>Bacterial_Wilt</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ralstonia solanacearum</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Root, Stem, Vascular</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>cucurbit yellow vine decline, Fusarium</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Leaf_Mosaic_Virus</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+          <t>Septoria_Leaf_Blotch</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Septoria lycopersici</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Fungal</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Foliar, Stem</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Circular, tan to gray lesions develop on the lower leaves and stems of the plant, typically smaller than 1/8 inch, but can multiply to cause entire leaf blight.. Small dark spots (pycnidia) in lesion centers where spores are produced; dark-brown perimeter with possible yellow halo; water-soaked appearance on leaf undersides; lesions are smaller than early blight and lack concentric rings; lesion centers do not crack open like gray leaf spot.. Early blight, Gray leaf spot</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Leaf_Yellow_Virus</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+          <t>Target_Spot</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Corynespora cassiicola</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fungal</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Root, Stem, Foliar, Fruit</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Leaf lesions are initially dark brown and pinpoint; as they enlarge, centers become light brown to gray with dark outer concentric rings sometimes surrounded by a diffuse yellowing (chlorosis). Fruit lesions start as small, brown, sunken flecks that expand into deeply pitted lesions with characteristic X or star-shaped cracking patterns.. Concentric ring pattern with light brown center and dark outer rings on leaf lesions; deeply pitted fruit lesions that develop during ripening; leaf lesions coalesce to cause blighting and premature defoliation; fruit lesions often develop on the side facing the interior canopy.. Bacterial spot, Early blight, Gray leaf spot</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mold_Leaf</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+          <t>Southern_Blight</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Athelia rolfsii</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Fungal</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Foliar, Stem, Root, Pod</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Initial water-soaked lesions on lower leaves and stems that progress to yellowing and wilting. Infection girdles the base of the stem at the soil line. White fungal mats develop on infected tissue with characteristic spherical resting structures (sclerotia) appearing on infected areas and soil.. Distinctive white fungal mats (mycelia) radiating from infected tissue onto the soil surface, and characteristic spherical sclerotia ranging in color from light tan to dark reddish-brown to black, approximately the size of mustard seeds; white cottony mycelium at the stem base.. White mold</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Mosaic_Virus</t>
+          <t>Phytophthora_Blight</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1029,44 +1129,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Two_Spotted_Spider_Mites_Leaf</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Yellow_Leaf_Curl_Virus</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>